<commit_message>
Saldo migratorio en personas: principal, Dentro de la region y nacional; periodo comunal de Migracion con guion
</commit_message>
<xml_diff>
--- a/output/graficos_regionales_migracion/plot_migracion_saldo_2019_antofagasta.xlsx
+++ b/output/graficos_regionales_migracion/plot_migracion_saldo_2019_antofagasta.xlsx
@@ -6,58 +6,120 @@
     <workbookView xWindow="0" yWindow="0" windowWidth="13125" windowHeight="6105" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Histórico" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Resumen" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Metadata" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Corrientes" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Composicion" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Histórico'!$A$1:$C$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Composicion'!$A$1:$C$11</definedName>
   </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="34">
+  <si>
+    <t xml:space="preserve">Saldo (personas)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Llegaron</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Se fueron</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Llegaron por cada 100 que se fueron</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fecha de creación</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-09-30 10:17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fuente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PIT - MDSF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Imagen asociada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">plot_migracion_saldo_2019_antofagasta.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Indicador</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M_SALDOMIGR_a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unidad territorial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Región de Antofagasta</t>
+  </si>
   <si>
     <t xml:space="preserve">Año</t>
   </si>
   <si>
-    <t xml:space="preserve">Saldo migratorio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Saldo acumulado</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Campo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Valor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fecha de creación</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-09-16 18:40</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fuente</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PIT - MDSF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Imagen asociada</t>
-  </si>
-  <si>
-    <t xml:space="preserve">plot_migracion_saldo_2019_antofagasta.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Indicador</t>
-  </si>
-  <si>
-    <t xml:space="preserve"/>
-  </si>
-  <si>
-    <t xml:space="preserve">Unidad territorial</t>
+    <t xml:space="preserve">2019</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Saldo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eje</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Grupo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nacionalidad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chilena</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Extranjera</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sin dato</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sexo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mujeres</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hombres</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tramo de edad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0 a 4 años</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5 a 14 años</t>
+  </si>
+  <si>
+    <t xml:space="preserve">15 a 29 años</t>
+  </si>
+  <si>
+    <t xml:space="preserve">30 a 59 años</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Desde 60 años</t>
   </si>
 </sst>
 </file>
@@ -422,9 +484,10 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="1" max="1" width="10.71" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="18.71" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="17.71" hidden="0" customWidth="1"/>
+    <col min="1" max="1" width="18.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="10.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="11.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="37.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -437,75 +500,26 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>2019</v>
+        <v>-1547</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>-1547</v>
+        <v>17691</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>-1547</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="n">
-        <v>2020</v>
-      </c>
-      <c r="B3" s="2" t="n">
-        <v>-4476</v>
-      </c>
-      <c r="C3" s="2" t="n">
-        <v>-6023</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="n">
-        <v>2021</v>
-      </c>
-      <c r="B4" s="2" t="n">
-        <v>-8875</v>
-      </c>
-      <c r="C4" s="2" t="n">
-        <v>-14898</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="n">
-        <v>2022</v>
-      </c>
-      <c r="B5" s="2" t="n">
-        <v>-4430</v>
-      </c>
-      <c r="C5" s="2" t="n">
-        <v>-19328</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="n">
-        <v>2023</v>
-      </c>
-      <c r="B6" s="2" t="n">
-        <v>-5880</v>
-      </c>
-      <c r="C6" s="2" t="n">
-        <v>-25208</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="n">
-        <v>2024</v>
-      </c>
-      <c r="B7" s="2" t="n">
-        <v>-5809</v>
-      </c>
-      <c r="C7" s="2" t="n">
-        <v>-31017</v>
+        <v>19238</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>92</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C7"/>
+  <autoFilter ref="A1:D2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
@@ -522,62 +536,316 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <cols>
+    <col min="1" max="1" width="10.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="10.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="11.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="10.71" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>2019</v>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>17691</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>19238</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>-1547</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2020</v>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>16779</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>21255</v>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>-4476</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>2021</v>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>19345</v>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>28220</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>-8875</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>2022</v>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>21208</v>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>25638</v>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>-4430</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>19857</v>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>25737</v>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>-5880</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>20652</v>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>26461</v>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>-5809</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:D7"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <cols>
+    <col min="1" max="1" width="15.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="15.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="18.71" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>-1766</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>-986</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>-561</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>-86</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>-119</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>-548</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>-582</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>-212</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:C11"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
 </file>
</xml_diff>